<commit_message>
Remove screenshot evidence references
</commit_message>
<xml_diff>
--- a/Hamid_Saleem_9061_Assignment4_BidLog.xlsx
+++ b/Hamid_Saleem_9061_Assignment4_BidLog.xlsx
@@ -863,7 +863,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Interested - requested sample screens</t>
+          <t>Interested - requested prototype outline</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>1 out of 2 responses (50%). The travel agency client showed interest and requested sample screens.</t>
+          <t>1 out of 2 responses (50%). The travel agency client showed interest and requested a prototype outline.</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>The Firebase chat module attracted a lot of competition. I should include a small screenshot or demo link for chat-related projects because clients need proof.</t>
+          <t>The Firebase chat module attracted a lot of competition. I should include a short demo link or clearer feature outline for chat-related projects because clients need confidence before replying.</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>On the final day I will bid earlier and choose projects where the first deliverable can be shown visually, because screenshots help new freelancers build trust.</t>
+          <t>On the final day I will bid earlier and choose projects where the first deliverable can be described clearly, because clear scope helps new freelancers build trust.</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>After this assignment, my strategy is to prepare reusable portfolio screenshots and place two focused bids every morning before competition increases.</t>
+          <t>After this assignment, my strategy is to prepare reusable portfolio descriptions and place two focused bids every morning before competition increases.</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>The best strategies were: keep the scope small, connect the app to the client's business, ask one smart question, bid early, and share relevant GitHub or screenshot evidence.</t>
+          <t>The best strategies were: keep the scope small, connect the app to the client's business, ask one smart question, bid early, and share a relevant GitHub link or project outline.</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Complete the Freelancer profile, verify GitHub link, pin mobile app repos, prepare screenshots, continue two bids per day, and build a simple portfolio website.</t>
+          <t>Complete the Freelancer profile, verify GitHub link, pin mobile app repos, prepare project descriptions, continue two bids per day, and build a simple portfolio website.</t>
         </is>
       </c>
     </row>

</xml_diff>